<commit_message>
fix(sample-data): rebuild SFY and PRIME exhibit files with proper 4-row header structure
Previous files were stubs with only a filler row. Exhibit files require 4
header rows (skipped by normalize_sfy_df/normalize_prime_df) followed by
column headers and data rows with loan programs matching MASTER_SHEET.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/data/sample/files_required/PRIME_02-18-2026_ExhibitAtoFormofSaleNotice - Pre-Funding.xlsx
+++ b/backend/data/sample/files_required/PRIME_02-18-2026_ExhibitAtoFormofSaleNotice - Pre-Funding.xlsx
@@ -413,56 +413,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Filler row 1</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr"/>
-      <c r="C1" t="inlineStr"/>
-      <c r="D1" t="inlineStr"/>
-      <c r="E1" t="inlineStr"/>
-      <c r="F1" t="inlineStr"/>
+          <t>Exhibit A - Pre-Funding</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Filler row 2</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
+          <t>Platform: PRIME</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Filler row 3</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
+      <c r="A3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Filler row 4</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
+      <c r="A4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -482,52 +454,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Orig. Balance</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Lender Price(%)</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Purchase Price</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>FICO Borrower</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>DTI</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>PTI</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Term</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>APR</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>Property State</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>Submit Date</t>
+          <t>TU144</t>
         </is>
       </c>
     </row>
@@ -544,48 +471,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>STANDARD</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>175000</v>
-      </c>
-      <c r="E6" t="n">
-        <v>98.5</v>
-      </c>
-      <c r="F6" t="n">
-        <v>172375</v>
-      </c>
-      <c r="G6" t="n">
-        <v>720</v>
-      </c>
-      <c r="H6" t="n">
-        <v>35</v>
-      </c>
-      <c r="I6" t="n">
-        <v>20</v>
-      </c>
-      <c r="J6" t="n">
-        <v>120</v>
-      </c>
-      <c r="K6" t="n">
-        <v>6.25</v>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>CA</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>2026-02-01</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SFC_2003</t>
+          <t>SFC_2002</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -595,93 +491,31 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>STANDARD</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>195000</v>
-      </c>
-      <c r="E7" t="n">
-        <v>98</v>
-      </c>
-      <c r="F7" t="n">
-        <v>191100</v>
-      </c>
-      <c r="G7" t="n">
-        <v>700</v>
-      </c>
-      <c r="H7" t="n">
-        <v>38</v>
-      </c>
-      <c r="I7" t="n">
-        <v>21</v>
-      </c>
-      <c r="J7" t="n">
-        <v>120</v>
-      </c>
-      <c r="K7" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>FL</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>2026-02-10</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SFC_2005</t>
+          <t>SFC_2003</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>FX3_PRIME_NEW</t>
+          <t>FX3_PRIME_HD</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>HD NOTE</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>310000</v>
-      </c>
-      <c r="E8" t="n">
-        <v>98.25</v>
-      </c>
-      <c r="F8" t="n">
-        <v>304575</v>
-      </c>
-      <c r="G8" t="n">
-        <v>750</v>
-      </c>
-      <c r="H8" t="n">
-        <v>32</v>
-      </c>
-      <c r="I8" t="n">
-        <v>18</v>
-      </c>
-      <c r="J8" t="n">
-        <v>120</v>
-      </c>
-      <c r="K8" t="n">
-        <v>6.1</v>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>WA</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>2026-02-12</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(sample-data): correct SFY/PRIME exhibit row offset (headers at pandas index 4)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/data/sample/files_required/PRIME_02-18-2026_ExhibitAtoFormofSaleNotice - Pre-Funding.xlsx
+++ b/backend/data/sample/files_required/PRIME_02-18-2026_ExhibitAtoFormofSaleNotice - Pre-Funding.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -437,51 +437,34 @@
       <c r="A4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>SELLER Loan #</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Loan Program</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Application Type</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>TU144</t>
-        </is>
-      </c>
+      <c r="A5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SFC_2001</t>
+          <t>SELLER Loan #</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>FX3_PRIME_STD</t>
+          <t>Loan Program</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>STANDARD</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>0</v>
+          <t>Application Type</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>TU144</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SFC_2002</t>
+          <t>SFC_2001</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -501,20 +484,40 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>SFC_2002</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>FX3_PRIME_STD</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>SFC_2003</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>FX3_PRIME_HD</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>HD NOTE</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="D9" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(sample-data): add underwriting columns to SFY/PRIME exhibit files
Added: Orig. Balance, Income, FICO Borrower, DTI, PTI, Stamp fee

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/data/sample/files_required/PRIME_02-18-2026_ExhibitAtoFormofSaleNotice - Pre-Funding.xlsx
+++ b/backend/data/sample/files_required/PRIME_02-18-2026_ExhibitAtoFormofSaleNotice - Pre-Funding.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -460,6 +460,36 @@
           <t>TU144</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Orig. Balance</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>FICO Borrower</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>DTI</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>PTI</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Stamp fee</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -480,6 +510,24 @@
       <c r="D7" t="n">
         <v>0</v>
       </c>
+      <c r="E7" t="n">
+        <v>200000</v>
+      </c>
+      <c r="F7" t="n">
+        <v>78000</v>
+      </c>
+      <c r="G7" t="n">
+        <v>710</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -500,6 +548,24 @@
       <c r="D8" t="n">
         <v>0</v>
       </c>
+      <c r="E8" t="n">
+        <v>165000</v>
+      </c>
+      <c r="F8" t="n">
+        <v>66000</v>
+      </c>
+      <c r="G8" t="n">
+        <v>695</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -518,6 +584,24 @@
         </is>
       </c>
       <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>290000</v>
+      </c>
+      <c r="F9" t="n">
+        <v>90000</v>
+      </c>
+      <c r="G9" t="n">
+        <v>730</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J9" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>